<commit_message>
Atualiza rodape (instagram/logo UFF) e Lattes/ORCID do Pedro Lima
</commit_message>
<xml_diff>
--- a/assets/img/team/team.xlsx
+++ b/assets/img/team/team.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/311e591e3f9068c5/Documentos/graphid/graphid-uff.github.io-main/assets/img/team/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="181" documentId="11_B7EDF1EB85707CAD8B3799FB57EF82E5A3543386" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0ADE17FE-70D9-4206-B68D-DD372B311E39}"/>
+  <xr:revisionPtr revIDLastSave="261" documentId="11_B7EDF1EB85707CAD8B3799FB57EF82E5A3543386" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{451114A3-5967-4574-808E-5E1804F43973}"/>
   <bookViews>
-    <workbookView xWindow="9630" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="104">
   <si>
     <t>Nome</t>
   </si>
@@ -182,9 +182,6 @@
     <t>Graduando</t>
   </si>
   <si>
-    <t>Linha de Pesquisa</t>
-  </si>
-  <si>
     <t>Descrição</t>
   </si>
   <si>
@@ -197,51 +194,21 @@
     <t>Redução e Mitigação de Risco de Desastres</t>
   </si>
   <si>
-    <t>Planejamento estratégico de ações preventivas e mitigadoras de risco de desastres, com foco em movimentos de massa em áreas prioritárias urbanas.</t>
-  </si>
-  <si>
-    <t>Mapeamento Colaborativo e Participação Comunitária</t>
-  </si>
-  <si>
-    <t>Levantamentos de campo e mapeamentos colaborativos com moradores de áreas de risco, valorizando a percepção e o conhecimento local como parte do diagnóstico técnico.</t>
-  </si>
-  <si>
-    <t>Educação, Autoproteção e Empoderamento Comunitário</t>
-  </si>
-  <si>
-    <t>Ações voltadas à capacitação e ao empoderamento das comunidades em risco, fortalecendo sua autonomia frente às informações e medidas de autoproteção.</t>
-  </si>
-  <si>
     <t>Conectividade Hidrossedimentológica</t>
   </si>
   <si>
-    <t>Hidrogeomorfologia de encostas e canais, zoneamento hidrossedimentológico (IHC) e validação da conectividade da paisagem.</t>
-  </si>
-  <si>
     <t>Uso e Cobertura do Solo (LULC)</t>
   </si>
   <si>
-    <t>Efeitos das mudanças de uso e cobertura do solo na perda de solo, na infiltração/escoamento/evapotranspiração e nas vazões.</t>
-  </si>
-  <si>
     <t>Mudanças Climáticas</t>
   </si>
   <si>
-    <t>Comportamento de eventos de precipitação extremos (intensidade, duração e frequência), tendência de vazões e tendências de chuva associadas a deslizamentos.</t>
-  </si>
-  <si>
     <t>Ocupação Territorial</t>
   </si>
   <si>
-    <t>Tendência de expansão urbana, suscetibilidade dos locais ocupados e modificação urbana do perigo.</t>
-  </si>
-  <si>
     <t>Sistema de Alerta</t>
   </si>
   <si>
-    <t>Limiares de precipitação e condições de deflagração, protocolos de acionamento e previsão de deslizamentos.</t>
-  </si>
-  <si>
     <t>Geotecnologias Aplicadas à Análise Espacial, Mapeamento e Modelagem de Perigo/Risco</t>
   </si>
   <si>
@@ -294,13 +261,85 @@
   </si>
   <si>
     <t>Pesquisador Colaborador</t>
+  </si>
+  <si>
+    <t>Área</t>
+  </si>
+  <si>
+    <t>Nome Origina, DOC Fran</t>
+  </si>
+  <si>
+    <t>Linha de Pesquisa (retrabalhado)</t>
+  </si>
+  <si>
+    <t>CONECTIVIDADE</t>
+  </si>
+  <si>
+    <t>LULC</t>
+  </si>
+  <si>
+    <t>PROCESSOS HIDROLÓGICOS</t>
+  </si>
+  <si>
+    <t>Fluxo de Água no Solo; Geração de Escoamento</t>
+  </si>
+  <si>
+    <t>Hidrogeomorfologia de Encostas e Canais eConectividade; IHC - Zoneamento Hidrossedimentológico; Validação da Conectividade</t>
+  </si>
+  <si>
+    <t>Efeito na Perda de Solo; Efeito naInfiltrção/Escoamento/ETP; Efeito nas Vazões</t>
+  </si>
+  <si>
+    <t>Comportamento de eventos de precipitação extretmos (i, d e f); Tendência de Vazões; Tendências de chuva para deslizamentos; Tendência de Desastres</t>
+  </si>
+  <si>
+    <t>DESASTRE</t>
+  </si>
+  <si>
+    <t>HIDROLOGIA</t>
+  </si>
+  <si>
+    <t>Tendência de Expansão; Suscetibilidade dos locaisocupados; Modificação Urbana do Perigo</t>
+  </si>
+  <si>
+    <t>Limiares precipitação/Condições deDeflagração; Protocolos; Previsão de Deslizamentos</t>
+  </si>
+  <si>
+    <t>MAPEAMENTO E MODELAGEM DE PERIGO/RISCO</t>
+  </si>
+  <si>
+    <t>Inventário de Deslizamentos; Inventário deEnxurradas/Alagamentos/Inundações; Modelagem de Estabilidade de Encostas</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - </t>
+  </si>
+  <si>
+    <t>Termos chave</t>
+  </si>
+  <si>
+    <t>Estudos de hidrogeomorfologia de encostas e canais, desenvolvimento e aplicação do Índice de Conectividade Hidrossedimentológica (IHC), zoneamento hidrossedimentológico e validação da conectividade da paisagem.</t>
+  </si>
+  <si>
+    <t>Avaliação dos efeitos das mudanças de uso e cobertura do solo sobre a perda de solo, a infiltração, o escoamento superficial, a evapotranspiração e as vazões em bacias hidrográficas.</t>
+  </si>
+  <si>
+    <t>Análise das tendências e do comportamento de eventos extremos de precipitação (intensidade, duração e frequência), das tendências de vazões, das condições de chuva associadas a deslizamentos e da evolução temporal dos desastres naturais.</t>
+  </si>
+  <si>
+    <t>Investigação das tendências de expansão territorial, da suscetibilidade das áreas ocupadas e das modificações do perigo decorrentes da urbanização e da ocupação do território.</t>
+  </si>
+  <si>
+    <t>Desenvolvimento de limiares de precipitação e condições de deflagração, protocolos de acionamento e modelos de previsão de deslizamentos para apoio a sistemas de alerta.</t>
+  </si>
+  <si>
+    <t>Desenvolvimento, avaliação e implementação de estratégias e medidas estruturais e não estruturais para redução e mitigação do risco de desastres, com foco na prevenção, no planejamento e no aumento da resiliência das áreas vulneráveis.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -326,6 +365,14 @@
       <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -381,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -393,6 +440,33 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -409,10 +483,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1012,10 +1082,10 @@
         <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -1137,230 +1207,274 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="70" customWidth="1"/>
-    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.6328125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="40" style="10" customWidth="1"/>
+    <col min="4" max="4" width="40" style="9" customWidth="1"/>
+    <col min="5" max="5" width="70" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="F1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="5" t="s">
+    </row>
+    <row r="2" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+      <c r="D2" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A3" s="6"/>
+      <c r="B3" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="6"/>
+      <c r="B4" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A5" s="6"/>
+      <c r="B5" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+    </row>
+    <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+    </row>
+    <row r="7" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="6"/>
+      <c r="B7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="A8" s="6"/>
+      <c r="B8" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="6"/>
+      <c r="B9" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-    </row>
-    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" spans="1:7" ht="58" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
+      <c r="D9" s="8"/>
+      <c r="E9" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-    </row>
-    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-    </row>
-    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "Atualiza rodape (instagram/logo UFF) e Lattes/ORCID do Pedro Lima"
This reverts commit 918dcc1e9a6e129a07b7fe2b1b6f423793f3f1b0.
</commit_message>
<xml_diff>
--- a/assets/img/team/team.xlsx
+++ b/assets/img/team/team.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/311e591e3f9068c5/Documentos/graphid/graphid-uff.github.io-main/assets/img/team/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="261" documentId="11_B7EDF1EB85707CAD8B3799FB57EF82E5A3543386" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{451114A3-5967-4574-808E-5E1804F43973}"/>
+  <xr:revisionPtr revIDLastSave="181" documentId="11_B7EDF1EB85707CAD8B3799FB57EF82E5A3543386" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0ADE17FE-70D9-4206-B68D-DD372B311E39}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9630" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="91">
   <si>
     <t>Nome</t>
   </si>
@@ -182,6 +182,9 @@
     <t>Graduando</t>
   </si>
   <si>
+    <t>Linha de Pesquisa</t>
+  </si>
+  <si>
     <t>Descrição</t>
   </si>
   <si>
@@ -194,21 +197,51 @@
     <t>Redução e Mitigação de Risco de Desastres</t>
   </si>
   <si>
+    <t>Planejamento estratégico de ações preventivas e mitigadoras de risco de desastres, com foco em movimentos de massa em áreas prioritárias urbanas.</t>
+  </si>
+  <si>
+    <t>Mapeamento Colaborativo e Participação Comunitária</t>
+  </si>
+  <si>
+    <t>Levantamentos de campo e mapeamentos colaborativos com moradores de áreas de risco, valorizando a percepção e o conhecimento local como parte do diagnóstico técnico.</t>
+  </si>
+  <si>
+    <t>Educação, Autoproteção e Empoderamento Comunitário</t>
+  </si>
+  <si>
+    <t>Ações voltadas à capacitação e ao empoderamento das comunidades em risco, fortalecendo sua autonomia frente às informações e medidas de autoproteção.</t>
+  </si>
+  <si>
     <t>Conectividade Hidrossedimentológica</t>
   </si>
   <si>
+    <t>Hidrogeomorfologia de encostas e canais, zoneamento hidrossedimentológico (IHC) e validação da conectividade da paisagem.</t>
+  </si>
+  <si>
     <t>Uso e Cobertura do Solo (LULC)</t>
   </si>
   <si>
+    <t>Efeitos das mudanças de uso e cobertura do solo na perda de solo, na infiltração/escoamento/evapotranspiração e nas vazões.</t>
+  </si>
+  <si>
     <t>Mudanças Climáticas</t>
   </si>
   <si>
+    <t>Comportamento de eventos de precipitação extremos (intensidade, duração e frequência), tendência de vazões e tendências de chuva associadas a deslizamentos.</t>
+  </si>
+  <si>
     <t>Ocupação Territorial</t>
   </si>
   <si>
+    <t>Tendência de expansão urbana, suscetibilidade dos locais ocupados e modificação urbana do perigo.</t>
+  </si>
+  <si>
     <t>Sistema de Alerta</t>
   </si>
   <si>
+    <t>Limiares de precipitação e condições de deflagração, protocolos de acionamento e previsão de deslizamentos.</t>
+  </si>
+  <si>
     <t>Geotecnologias Aplicadas à Análise Espacial, Mapeamento e Modelagem de Perigo/Risco</t>
   </si>
   <si>
@@ -261,85 +294,13 @@
   </si>
   <si>
     <t>Pesquisador Colaborador</t>
-  </si>
-  <si>
-    <t>Área</t>
-  </si>
-  <si>
-    <t>Nome Origina, DOC Fran</t>
-  </si>
-  <si>
-    <t>Linha de Pesquisa (retrabalhado)</t>
-  </si>
-  <si>
-    <t>CONECTIVIDADE</t>
-  </si>
-  <si>
-    <t>LULC</t>
-  </si>
-  <si>
-    <t>PROCESSOS HIDROLÓGICOS</t>
-  </si>
-  <si>
-    <t>Fluxo de Água no Solo; Geração de Escoamento</t>
-  </si>
-  <si>
-    <t>Hidrogeomorfologia de Encostas e Canais eConectividade; IHC - Zoneamento Hidrossedimentológico; Validação da Conectividade</t>
-  </si>
-  <si>
-    <t>Efeito na Perda de Solo; Efeito naInfiltrção/Escoamento/ETP; Efeito nas Vazões</t>
-  </si>
-  <si>
-    <t>Comportamento de eventos de precipitação extretmos (i, d e f); Tendência de Vazões; Tendências de chuva para deslizamentos; Tendência de Desastres</t>
-  </si>
-  <si>
-    <t>DESASTRE</t>
-  </si>
-  <si>
-    <t>HIDROLOGIA</t>
-  </si>
-  <si>
-    <t>Tendência de Expansão; Suscetibilidade dos locaisocupados; Modificação Urbana do Perigo</t>
-  </si>
-  <si>
-    <t>Limiares precipitação/Condições deDeflagração; Protocolos; Previsão de Deslizamentos</t>
-  </si>
-  <si>
-    <t>MAPEAMENTO E MODELAGEM DE PERIGO/RISCO</t>
-  </si>
-  <si>
-    <t>Inventário de Deslizamentos; Inventário deEnxurradas/Alagamentos/Inundações; Modelagem de Estabilidade de Encostas</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> - </t>
-  </si>
-  <si>
-    <t>Termos chave</t>
-  </si>
-  <si>
-    <t>Estudos de hidrogeomorfologia de encostas e canais, desenvolvimento e aplicação do Índice de Conectividade Hidrossedimentológica (IHC), zoneamento hidrossedimentológico e validação da conectividade da paisagem.</t>
-  </si>
-  <si>
-    <t>Avaliação dos efeitos das mudanças de uso e cobertura do solo sobre a perda de solo, a infiltração, o escoamento superficial, a evapotranspiração e as vazões em bacias hidrográficas.</t>
-  </si>
-  <si>
-    <t>Análise das tendências e do comportamento de eventos extremos de precipitação (intensidade, duração e frequência), das tendências de vazões, das condições de chuva associadas a deslizamentos e da evolução temporal dos desastres naturais.</t>
-  </si>
-  <si>
-    <t>Investigação das tendências de expansão territorial, da suscetibilidade das áreas ocupadas e das modificações do perigo decorrentes da urbanização e da ocupação do território.</t>
-  </si>
-  <si>
-    <t>Desenvolvimento de limiares de precipitação e condições de deflagração, protocolos de acionamento e modelos de previsão de deslizamentos para apoio a sistemas de alerta.</t>
-  </si>
-  <si>
-    <t>Desenvolvimento, avaliação e implementação de estratégias e medidas estruturais e não estruturais para redução e mitigação do risco de desastres, com foco na prevenção, no planejamento e no aumento da resiliência das áreas vulneráveis.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -365,14 +326,6 @@
       <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -428,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -440,33 +393,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,6 +409,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1082,10 +1012,10 @@
         <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -1207,274 +1137,230 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.6328125" style="10" customWidth="1"/>
-    <col min="3" max="3" width="40" style="10" customWidth="1"/>
-    <col min="4" max="4" width="40" style="9" customWidth="1"/>
-    <col min="5" max="5" width="70" customWidth="1"/>
-    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="70" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="11" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C1" s="7" t="s">
+    </row>
+    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D1" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="F8" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" s="8" t="s">
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A3" s="6"/>
-      <c r="B3" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" s="8" t="s">
+      <c r="E11" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="6"/>
-      <c r="B4" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="8" t="s">
+      <c r="F11" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A5" s="6"/>
-      <c r="B5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-    </row>
-    <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-    </row>
-    <row r="7" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="6"/>
-      <c r="B7" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="J7" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" s="6"/>
-      <c r="B8" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="6"/>
-      <c r="B9" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dados do André na equipe com Lattes, ORCID e palavras-chave reais
</commit_message>
<xml_diff>
--- a/assets/img/team/team.xlsx
+++ b/assets/img/team/team.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/311e591e3f9068c5/Documentos/graphid/graphid-uff.github.io-main/assets/img/team/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_DBB540A7EB1D52A5B7CC033F56D0052E45279F2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2254153-639C-42EF-B642-E3E60BED35B9}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_DBB540A7EB1D52A5B7CC033F56D0052E45279F2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{622B5D3D-2CAF-4864-BDC8-0DFA34E972A0}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="7470" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="270">
   <si>
     <t>Nome</t>
   </si>
@@ -887,6 +887,45 @@
     <t xml:space="preserve">O inventário de deslizamentos do município do Rio de Janeiro baseia-se, predominantemente, em ocorrências reportadas pela população, o que introduz um viés em favor de áreas ocupadas e limita a representação de deslizamentos naturais. O mapeamento histórico de cicatrizes em ambientes naturais busca reduzir essa limitação, ampliando a representatividade do inventário e permitindo o desenvolvimento de modelos de suscetibilidade mais robustos, além de contribuir para uma melhor compreensão da dinâmica geomorfológica do município.
 </t>
   </si>
+  <si>
+    <t>Andre de Freitas Pimentel dos Anjos</t>
+  </si>
+  <si>
+    <t>http://lattes.cnpq.br/7795895409074741</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0009-0001-1983-7797</t>
+  </si>
+  <si>
+    <t>Previsão de Deslizamentos</t>
+  </si>
+  <si>
+    <t>Cereto et al., 2026</t>
+  </si>
+  <si>
+    <t>https://www.uff.br/</t>
+  </si>
+  <si>
+    <t>Sem DOI localizado</t>
+  </si>
+  <si>
+    <t>Use of Random Forest Classifier for the Prediction of Landslide-Related Occurrences in Petrópolis, RJ, Brazil</t>
+  </si>
+  <si>
+    <t>10º Workshop em Engenharia de Biossistemas (WEB 10.0) – PGEB/UFF</t>
+  </si>
+  <si>
+    <t>Anjos et al., 2025</t>
+  </si>
+  <si>
+    <t>https://ojs.celsotech.io/index.php/revista/issue/view/12</t>
+  </si>
+  <si>
+    <t>Anais do IV SETEC RRD RIO</t>
+  </si>
+  <si>
+    <t>Revista Presença – Anais do IV SETEC RRD RIO</t>
+  </si>
 </sst>
 </file>
 
@@ -895,7 +934,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mmmm/yyyy"/>
   </numFmts>
-  <fonts count="42">
+  <fonts count="43">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1138,8 +1177,13 @@
       <color rgb="FF1155CC"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1186,6 +1230,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFA61C00"/>
         <bgColor rgb="FFA61C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEAF1"/>
       </patternFill>
     </fill>
   </fills>
@@ -1286,7 +1335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1441,6 +1490,10 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1449,15 +1502,21 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1474,6 +1533,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1944,24 +2007,38 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="14.25" customHeight="1">
-      <c r="A8" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="11" t="s">
+    <row r="8" spans="1:11" s="79" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A8" s="53" t="s">
+        <v>257</v>
+      </c>
+      <c r="B8" s="53" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="D8" s="46"/>
-      <c r="E8" s="46"/>
-      <c r="F8" s="46"/>
-      <c r="G8" s="46"/>
-      <c r="H8" s="46"/>
-      <c r="I8" s="46"/>
-      <c r="J8" s="46"/>
-      <c r="K8" s="46"/>
+      <c r="D8" s="78" t="s">
+        <v>258</v>
+      </c>
+      <c r="E8" s="78" t="s">
+        <v>259</v>
+      </c>
+      <c r="F8" s="78"/>
+      <c r="G8" s="78" t="s">
+        <v>156</v>
+      </c>
+      <c r="H8" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="I8" s="78" t="s">
+        <v>260</v>
+      </c>
+      <c r="J8" s="78" t="s">
+        <v>117</v>
+      </c>
+      <c r="K8" s="78" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="14.25" customHeight="1">
       <c r="A9" s="11" t="s">
@@ -9272,18 +9349,18 @@
       <c r="E1" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="68" t="s">
+      <c r="F1" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="70"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="72"/>
     </row>
     <row r="2" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="73" t="s">
         <v>44</v>
       </c>
       <c r="B2" s="14" t="s">
@@ -9316,7 +9393,7 @@
       <c r="K2" s="20"/>
     </row>
     <row r="3" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A3" s="72"/>
+      <c r="A3" s="74"/>
       <c r="B3" s="14" t="s">
         <v>63</v>
       </c>
@@ -9347,7 +9424,7 @@
       <c r="K3" s="20"/>
     </row>
     <row r="4" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A4" s="72"/>
+      <c r="A4" s="74"/>
       <c r="B4" s="14" t="s">
         <v>77</v>
       </c>
@@ -9378,7 +9455,7 @@
       <c r="K4" s="20"/>
     </row>
     <row r="5" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A5" s="72"/>
+      <c r="A5" s="74"/>
       <c r="B5" s="24" t="s">
         <v>87</v>
       </c>
@@ -9405,7 +9482,7 @@
       <c r="K5" s="20"/>
     </row>
     <row r="6" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A6" s="73"/>
+      <c r="A6" s="75"/>
       <c r="B6" s="26" t="s">
         <v>93</v>
       </c>
@@ -9428,7 +9505,7 @@
       <c r="K6" s="20"/>
     </row>
     <row r="7" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A7" s="71" t="s">
+      <c r="A7" s="73" t="s">
         <v>100</v>
       </c>
       <c r="B7" s="24" t="s">
@@ -9459,7 +9536,7 @@
       <c r="K7" s="20"/>
     </row>
     <row r="8" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A8" s="72"/>
+      <c r="A8" s="74"/>
       <c r="B8" s="24" t="s">
         <v>110</v>
       </c>
@@ -9490,7 +9567,7 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A9" s="72"/>
+      <c r="A9" s="74"/>
       <c r="B9" s="32" t="s">
         <v>118</v>
       </c>
@@ -9521,7 +9598,7 @@
       <c r="K9" s="20"/>
     </row>
     <row r="10" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A10" s="72"/>
+      <c r="A10" s="74"/>
       <c r="B10" s="14" t="s">
         <v>131</v>
       </c>
@@ -9546,7 +9623,7 @@
       <c r="K10" s="20"/>
     </row>
     <row r="11" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A11" s="72"/>
+      <c r="A11" s="74"/>
       <c r="B11" s="35" t="s">
         <v>137</v>
       </c>
@@ -15691,12 +15768,12 @@
   <sheetData>
     <row r="1" spans="1:27">
       <c r="A1" s="1"/>
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
@@ -16191,14 +16268,24 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27">
-      <c r="A14" s="9">
+      <c r="A14" s="80">
         <v>12</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
+      <c r="B14" s="81" t="s">
+        <v>261</v>
+      </c>
+      <c r="C14" s="81" t="s">
+        <v>262</v>
+      </c>
+      <c r="D14" s="81" t="s">
+        <v>263</v>
+      </c>
+      <c r="E14" s="81" t="s">
+        <v>264</v>
+      </c>
+      <c r="F14" s="81" t="s">
+        <v>265</v>
+      </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -16222,14 +16309,24 @@
       <c r="AA14" s="3"/>
     </row>
     <row r="15" spans="1:27">
-      <c r="A15" s="9">
+      <c r="A15" s="80">
         <v>13</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
+      <c r="B15" s="81" t="s">
+        <v>266</v>
+      </c>
+      <c r="C15" s="81" t="s">
+        <v>267</v>
+      </c>
+      <c r="D15" s="81" t="s">
+        <v>263</v>
+      </c>
+      <c r="E15" s="81" t="s">
+        <v>268</v>
+      </c>
+      <c r="F15" s="81" t="s">
+        <v>269</v>
+      </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -44869,11 +44966,11 @@
       <c r="B1" s="76" t="s">
         <v>229</v>
       </c>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
@@ -44983,11 +45080,11 @@
       <c r="B13" s="77" t="s">
         <v>243</v>
       </c>
-      <c r="C13" s="75"/>
-      <c r="D13" s="75"/>
-      <c r="E13" s="75"/>
-      <c r="F13" s="75"/>
-      <c r="G13" s="75"/>
+      <c r="C13" s="69"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="69"/>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="8" t="s">

</xml_diff>

<commit_message>
Deploying to gh-pages from @ graphid-uff/graphid-uff.github.io@75bb028a45c0650c7efc71626b4b4a392babb31c 🚀
</commit_message>
<xml_diff>
--- a/assets/img/team/team.xlsx
+++ b/assets/img/team/team.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/311e591e3f9068c5/Documentos/graphid/graphid-uff.github.io-main/assets/img/team/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_DBB540A7EB1D52A5B7CC033F56D0052E45279F2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2254153-639C-42EF-B642-E3E60BED35B9}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_DBB540A7EB1D52A5B7CC033F56D0052E45279F2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{622B5D3D-2CAF-4864-BDC8-0DFA34E972A0}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="7470" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="270">
   <si>
     <t>Nome</t>
   </si>
@@ -887,6 +887,45 @@
     <t xml:space="preserve">O inventário de deslizamentos do município do Rio de Janeiro baseia-se, predominantemente, em ocorrências reportadas pela população, o que introduz um viés em favor de áreas ocupadas e limita a representação de deslizamentos naturais. O mapeamento histórico de cicatrizes em ambientes naturais busca reduzir essa limitação, ampliando a representatividade do inventário e permitindo o desenvolvimento de modelos de suscetibilidade mais robustos, além de contribuir para uma melhor compreensão da dinâmica geomorfológica do município.
 </t>
   </si>
+  <si>
+    <t>Andre de Freitas Pimentel dos Anjos</t>
+  </si>
+  <si>
+    <t>http://lattes.cnpq.br/7795895409074741</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0009-0001-1983-7797</t>
+  </si>
+  <si>
+    <t>Previsão de Deslizamentos</t>
+  </si>
+  <si>
+    <t>Cereto et al., 2026</t>
+  </si>
+  <si>
+    <t>https://www.uff.br/</t>
+  </si>
+  <si>
+    <t>Sem DOI localizado</t>
+  </si>
+  <si>
+    <t>Use of Random Forest Classifier for the Prediction of Landslide-Related Occurrences in Petrópolis, RJ, Brazil</t>
+  </si>
+  <si>
+    <t>10º Workshop em Engenharia de Biossistemas (WEB 10.0) – PGEB/UFF</t>
+  </si>
+  <si>
+    <t>Anjos et al., 2025</t>
+  </si>
+  <si>
+    <t>https://ojs.celsotech.io/index.php/revista/issue/view/12</t>
+  </si>
+  <si>
+    <t>Anais do IV SETEC RRD RIO</t>
+  </si>
+  <si>
+    <t>Revista Presença – Anais do IV SETEC RRD RIO</t>
+  </si>
 </sst>
 </file>
 
@@ -895,7 +934,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mmmm/yyyy"/>
   </numFmts>
-  <fonts count="42">
+  <fonts count="43">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1138,8 +1177,13 @@
       <color rgb="FF1155CC"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1186,6 +1230,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFA61C00"/>
         <bgColor rgb="FFA61C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEAF1"/>
       </patternFill>
     </fill>
   </fills>
@@ -1286,7 +1335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1441,6 +1490,10 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1449,15 +1502,21 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1474,6 +1533,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1944,24 +2007,38 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="14.25" customHeight="1">
-      <c r="A8" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="11" t="s">
+    <row r="8" spans="1:11" s="79" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A8" s="53" t="s">
+        <v>257</v>
+      </c>
+      <c r="B8" s="53" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="D8" s="46"/>
-      <c r="E8" s="46"/>
-      <c r="F8" s="46"/>
-      <c r="G8" s="46"/>
-      <c r="H8" s="46"/>
-      <c r="I8" s="46"/>
-      <c r="J8" s="46"/>
-      <c r="K8" s="46"/>
+      <c r="D8" s="78" t="s">
+        <v>258</v>
+      </c>
+      <c r="E8" s="78" t="s">
+        <v>259</v>
+      </c>
+      <c r="F8" s="78"/>
+      <c r="G8" s="78" t="s">
+        <v>156</v>
+      </c>
+      <c r="H8" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="I8" s="78" t="s">
+        <v>260</v>
+      </c>
+      <c r="J8" s="78" t="s">
+        <v>117</v>
+      </c>
+      <c r="K8" s="78" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="14.25" customHeight="1">
       <c r="A9" s="11" t="s">
@@ -9272,18 +9349,18 @@
       <c r="E1" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="68" t="s">
+      <c r="F1" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="70"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="72"/>
     </row>
     <row r="2" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="73" t="s">
         <v>44</v>
       </c>
       <c r="B2" s="14" t="s">
@@ -9316,7 +9393,7 @@
       <c r="K2" s="20"/>
     </row>
     <row r="3" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A3" s="72"/>
+      <c r="A3" s="74"/>
       <c r="B3" s="14" t="s">
         <v>63</v>
       </c>
@@ -9347,7 +9424,7 @@
       <c r="K3" s="20"/>
     </row>
     <row r="4" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A4" s="72"/>
+      <c r="A4" s="74"/>
       <c r="B4" s="14" t="s">
         <v>77</v>
       </c>
@@ -9378,7 +9455,7 @@
       <c r="K4" s="20"/>
     </row>
     <row r="5" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A5" s="72"/>
+      <c r="A5" s="74"/>
       <c r="B5" s="24" t="s">
         <v>87</v>
       </c>
@@ -9405,7 +9482,7 @@
       <c r="K5" s="20"/>
     </row>
     <row r="6" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A6" s="73"/>
+      <c r="A6" s="75"/>
       <c r="B6" s="26" t="s">
         <v>93</v>
       </c>
@@ -9428,7 +9505,7 @@
       <c r="K6" s="20"/>
     </row>
     <row r="7" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A7" s="71" t="s">
+      <c r="A7" s="73" t="s">
         <v>100</v>
       </c>
       <c r="B7" s="24" t="s">
@@ -9459,7 +9536,7 @@
       <c r="K7" s="20"/>
     </row>
     <row r="8" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A8" s="72"/>
+      <c r="A8" s="74"/>
       <c r="B8" s="24" t="s">
         <v>110</v>
       </c>
@@ -9490,7 +9567,7 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A9" s="72"/>
+      <c r="A9" s="74"/>
       <c r="B9" s="32" t="s">
         <v>118</v>
       </c>
@@ -9521,7 +9598,7 @@
       <c r="K9" s="20"/>
     </row>
     <row r="10" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A10" s="72"/>
+      <c r="A10" s="74"/>
       <c r="B10" s="14" t="s">
         <v>131</v>
       </c>
@@ -9546,7 +9623,7 @@
       <c r="K10" s="20"/>
     </row>
     <row r="11" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A11" s="72"/>
+      <c r="A11" s="74"/>
       <c r="B11" s="35" t="s">
         <v>137</v>
       </c>
@@ -15691,12 +15768,12 @@
   <sheetData>
     <row r="1" spans="1:27">
       <c r="A1" s="1"/>
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
@@ -16191,14 +16268,24 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27">
-      <c r="A14" s="9">
+      <c r="A14" s="80">
         <v>12</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
+      <c r="B14" s="81" t="s">
+        <v>261</v>
+      </c>
+      <c r="C14" s="81" t="s">
+        <v>262</v>
+      </c>
+      <c r="D14" s="81" t="s">
+        <v>263</v>
+      </c>
+      <c r="E14" s="81" t="s">
+        <v>264</v>
+      </c>
+      <c r="F14" s="81" t="s">
+        <v>265</v>
+      </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -16222,14 +16309,24 @@
       <c r="AA14" s="3"/>
     </row>
     <row r="15" spans="1:27">
-      <c r="A15" s="9">
+      <c r="A15" s="80">
         <v>13</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
+      <c r="B15" s="81" t="s">
+        <v>266</v>
+      </c>
+      <c r="C15" s="81" t="s">
+        <v>267</v>
+      </c>
+      <c r="D15" s="81" t="s">
+        <v>263</v>
+      </c>
+      <c r="E15" s="81" t="s">
+        <v>268</v>
+      </c>
+      <c r="F15" s="81" t="s">
+        <v>269</v>
+      </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -44869,11 +44966,11 @@
       <c r="B1" s="76" t="s">
         <v>229</v>
       </c>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
@@ -44983,11 +45080,11 @@
       <c r="B13" s="77" t="s">
         <v>243</v>
       </c>
-      <c r="C13" s="75"/>
-      <c r="D13" s="75"/>
-      <c r="E13" s="75"/>
-      <c r="F13" s="75"/>
-      <c r="G13" s="75"/>
+      <c r="C13" s="69"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="69"/>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="8" t="s">

</xml_diff>

<commit_message>
Atualiza foto da Danúbia e ajusta enquadramento do rosto no card
</commit_message>
<xml_diff>
--- a/assets/img/team/team.xlsx
+++ b/assets/img/team/team.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/311e591e3f9068c5/Documentos/graphid/graphid-uff.github.io-main/assets/img/team/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_DBB540A7EB1D52A5B7CC033F56D0052E45279F2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{622B5D3D-2CAF-4864-BDC8-0DFA34E972A0}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_DBB540A7EB1D52A5B7CC033F56D0052E45279F2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89089B6F-1121-4683-9055-F11CCC5416C6}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="7470" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team" sheetId="1" r:id="rId1"/>
@@ -1490,6 +1490,16 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1507,16 +1517,6 @@
     </xf>
     <xf numFmtId="0" fontId="35" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2007,7 +2007,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:11" s="79" customFormat="1" ht="14.25" customHeight="1">
+    <row r="8" spans="1:11" s="69" customFormat="1" ht="14.25" customHeight="1">
       <c r="A8" s="53" t="s">
         <v>257</v>
       </c>
@@ -2017,26 +2017,26 @@
       <c r="C8" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="D8" s="78" t="s">
+      <c r="D8" s="68" t="s">
         <v>258</v>
       </c>
-      <c r="E8" s="78" t="s">
+      <c r="E8" s="68" t="s">
         <v>259</v>
       </c>
-      <c r="F8" s="78"/>
-      <c r="G8" s="78" t="s">
+      <c r="F8" s="68"/>
+      <c r="G8" s="68" t="s">
         <v>156</v>
       </c>
-      <c r="H8" s="78" t="s">
+      <c r="H8" s="68" t="s">
         <v>110</v>
       </c>
-      <c r="I8" s="78" t="s">
+      <c r="I8" s="68" t="s">
         <v>260</v>
       </c>
-      <c r="J8" s="78" t="s">
+      <c r="J8" s="68" t="s">
         <v>117</v>
       </c>
-      <c r="K8" s="78" t="s">
+      <c r="K8" s="68" t="s">
         <v>123</v>
       </c>
     </row>
@@ -9349,18 +9349,18 @@
       <c r="E1" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="70" t="s">
+      <c r="F1" s="74" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="72"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="76"/>
     </row>
     <row r="2" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="77" t="s">
         <v>44</v>
       </c>
       <c r="B2" s="14" t="s">
@@ -9393,7 +9393,7 @@
       <c r="K2" s="20"/>
     </row>
     <row r="3" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A3" s="74"/>
+      <c r="A3" s="78"/>
       <c r="B3" s="14" t="s">
         <v>63</v>
       </c>
@@ -9424,7 +9424,7 @@
       <c r="K3" s="20"/>
     </row>
     <row r="4" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A4" s="74"/>
+      <c r="A4" s="78"/>
       <c r="B4" s="14" t="s">
         <v>77</v>
       </c>
@@ -9455,7 +9455,7 @@
       <c r="K4" s="20"/>
     </row>
     <row r="5" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A5" s="74"/>
+      <c r="A5" s="78"/>
       <c r="B5" s="24" t="s">
         <v>87</v>
       </c>
@@ -9482,7 +9482,7 @@
       <c r="K5" s="20"/>
     </row>
     <row r="6" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A6" s="75"/>
+      <c r="A6" s="79"/>
       <c r="B6" s="26" t="s">
         <v>93</v>
       </c>
@@ -9505,7 +9505,7 @@
       <c r="K6" s="20"/>
     </row>
     <row r="7" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="77" t="s">
         <v>100</v>
       </c>
       <c r="B7" s="24" t="s">
@@ -9536,7 +9536,7 @@
       <c r="K7" s="20"/>
     </row>
     <row r="8" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A8" s="74"/>
+      <c r="A8" s="78"/>
       <c r="B8" s="24" t="s">
         <v>110</v>
       </c>
@@ -9567,7 +9567,7 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A9" s="74"/>
+      <c r="A9" s="78"/>
       <c r="B9" s="32" t="s">
         <v>118</v>
       </c>
@@ -9598,7 +9598,7 @@
       <c r="K9" s="20"/>
     </row>
     <row r="10" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A10" s="74"/>
+      <c r="A10" s="78"/>
       <c r="B10" s="14" t="s">
         <v>131</v>
       </c>
@@ -9623,7 +9623,7 @@
       <c r="K10" s="20"/>
     </row>
     <row r="11" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A11" s="74"/>
+      <c r="A11" s="78"/>
       <c r="B11" s="35" t="s">
         <v>137</v>
       </c>
@@ -15768,12 +15768,12 @@
   <sheetData>
     <row r="1" spans="1:27">
       <c r="A1" s="1"/>
-      <c r="B1" s="68" t="s">
+      <c r="B1" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
@@ -16268,22 +16268,22 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27">
-      <c r="A14" s="80">
+      <c r="A14" s="70">
         <v>12</v>
       </c>
-      <c r="B14" s="81" t="s">
+      <c r="B14" s="71" t="s">
         <v>261</v>
       </c>
-      <c r="C14" s="81" t="s">
+      <c r="C14" s="71" t="s">
         <v>262</v>
       </c>
-      <c r="D14" s="81" t="s">
+      <c r="D14" s="71" t="s">
         <v>263</v>
       </c>
-      <c r="E14" s="81" t="s">
+      <c r="E14" s="71" t="s">
         <v>264</v>
       </c>
-      <c r="F14" s="81" t="s">
+      <c r="F14" s="9" t="s">
         <v>265</v>
       </c>
       <c r="G14" s="3"/>
@@ -16309,22 +16309,22 @@
       <c r="AA14" s="3"/>
     </row>
     <row r="15" spans="1:27">
-      <c r="A15" s="80">
+      <c r="A15" s="70">
         <v>13</v>
       </c>
-      <c r="B15" s="81" t="s">
+      <c r="B15" s="71" t="s">
         <v>266</v>
       </c>
-      <c r="C15" s="81" t="s">
+      <c r="C15" s="71" t="s">
         <v>267</v>
       </c>
-      <c r="D15" s="81" t="s">
+      <c r="D15" s="71" t="s">
         <v>263</v>
       </c>
-      <c r="E15" s="81" t="s">
+      <c r="E15" s="71" t="s">
         <v>268</v>
       </c>
-      <c r="F15" s="81" t="s">
+      <c r="F15" s="9" t="s">
         <v>269</v>
       </c>
       <c r="G15" s="3"/>
@@ -44963,14 +44963,14 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="58"/>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="80" t="s">
         <v>229</v>
       </c>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
@@ -45077,14 +45077,14 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="62"/>
-      <c r="B13" s="77" t="s">
+      <c r="B13" s="81" t="s">
         <v>243</v>
       </c>
-      <c r="C13" s="69"/>
-      <c r="D13" s="69"/>
-      <c r="E13" s="69"/>
-      <c r="F13" s="69"/>
-      <c r="G13" s="69"/>
+      <c r="C13" s="73"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="73"/>
+      <c r="F13" s="73"/>
+      <c r="G13" s="73"/>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="8" t="s">

</xml_diff>

<commit_message>
Deploying to gh-pages from @ graphid-uff/graphid-uff.github.io@4694eab22dbee9ba66193132e298355ce6ded92c 🚀
</commit_message>
<xml_diff>
--- a/assets/img/team/team.xlsx
+++ b/assets/img/team/team.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/311e591e3f9068c5/Documentos/graphid/graphid-uff.github.io-main/assets/img/team/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_DBB540A7EB1D52A5B7CC033F56D0052E45279F2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{622B5D3D-2CAF-4864-BDC8-0DFA34E972A0}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_DBB540A7EB1D52A5B7CC033F56D0052E45279F2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89089B6F-1121-4683-9055-F11CCC5416C6}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="7470" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team" sheetId="1" r:id="rId1"/>
@@ -1490,6 +1490,16 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1507,16 +1517,6 @@
     </xf>
     <xf numFmtId="0" fontId="35" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2007,7 +2007,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:11" s="79" customFormat="1" ht="14.25" customHeight="1">
+    <row r="8" spans="1:11" s="69" customFormat="1" ht="14.25" customHeight="1">
       <c r="A8" s="53" t="s">
         <v>257</v>
       </c>
@@ -2017,26 +2017,26 @@
       <c r="C8" s="53" t="s">
         <v>175</v>
       </c>
-      <c r="D8" s="78" t="s">
+      <c r="D8" s="68" t="s">
         <v>258</v>
       </c>
-      <c r="E8" s="78" t="s">
+      <c r="E8" s="68" t="s">
         <v>259</v>
       </c>
-      <c r="F8" s="78"/>
-      <c r="G8" s="78" t="s">
+      <c r="F8" s="68"/>
+      <c r="G8" s="68" t="s">
         <v>156</v>
       </c>
-      <c r="H8" s="78" t="s">
+      <c r="H8" s="68" t="s">
         <v>110</v>
       </c>
-      <c r="I8" s="78" t="s">
+      <c r="I8" s="68" t="s">
         <v>260</v>
       </c>
-      <c r="J8" s="78" t="s">
+      <c r="J8" s="68" t="s">
         <v>117</v>
       </c>
-      <c r="K8" s="78" t="s">
+      <c r="K8" s="68" t="s">
         <v>123</v>
       </c>
     </row>
@@ -9349,18 +9349,18 @@
       <c r="E1" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="70" t="s">
+      <c r="F1" s="74" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="72"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="76"/>
     </row>
     <row r="2" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="77" t="s">
         <v>44</v>
       </c>
       <c r="B2" s="14" t="s">
@@ -9393,7 +9393,7 @@
       <c r="K2" s="20"/>
     </row>
     <row r="3" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A3" s="74"/>
+      <c r="A3" s="78"/>
       <c r="B3" s="14" t="s">
         <v>63</v>
       </c>
@@ -9424,7 +9424,7 @@
       <c r="K3" s="20"/>
     </row>
     <row r="4" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A4" s="74"/>
+      <c r="A4" s="78"/>
       <c r="B4" s="14" t="s">
         <v>77</v>
       </c>
@@ -9455,7 +9455,7 @@
       <c r="K4" s="20"/>
     </row>
     <row r="5" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A5" s="74"/>
+      <c r="A5" s="78"/>
       <c r="B5" s="24" t="s">
         <v>87</v>
       </c>
@@ -9482,7 +9482,7 @@
       <c r="K5" s="20"/>
     </row>
     <row r="6" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A6" s="75"/>
+      <c r="A6" s="79"/>
       <c r="B6" s="26" t="s">
         <v>93</v>
       </c>
@@ -9505,7 +9505,7 @@
       <c r="K6" s="20"/>
     </row>
     <row r="7" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="77" t="s">
         <v>100</v>
       </c>
       <c r="B7" s="24" t="s">
@@ -9536,7 +9536,7 @@
       <c r="K7" s="20"/>
     </row>
     <row r="8" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A8" s="74"/>
+      <c r="A8" s="78"/>
       <c r="B8" s="24" t="s">
         <v>110</v>
       </c>
@@ -9567,7 +9567,7 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A9" s="74"/>
+      <c r="A9" s="78"/>
       <c r="B9" s="32" t="s">
         <v>118</v>
       </c>
@@ -9598,7 +9598,7 @@
       <c r="K9" s="20"/>
     </row>
     <row r="10" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A10" s="74"/>
+      <c r="A10" s="78"/>
       <c r="B10" s="14" t="s">
         <v>131</v>
       </c>
@@ -9623,7 +9623,7 @@
       <c r="K10" s="20"/>
     </row>
     <row r="11" spans="1:12" ht="14.25" customHeight="1">
-      <c r="A11" s="74"/>
+      <c r="A11" s="78"/>
       <c r="B11" s="35" t="s">
         <v>137</v>
       </c>
@@ -15768,12 +15768,12 @@
   <sheetData>
     <row r="1" spans="1:27">
       <c r="A1" s="1"/>
-      <c r="B1" s="68" t="s">
+      <c r="B1" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
@@ -16268,22 +16268,22 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27">
-      <c r="A14" s="80">
+      <c r="A14" s="70">
         <v>12</v>
       </c>
-      <c r="B14" s="81" t="s">
+      <c r="B14" s="71" t="s">
         <v>261</v>
       </c>
-      <c r="C14" s="81" t="s">
+      <c r="C14" s="71" t="s">
         <v>262</v>
       </c>
-      <c r="D14" s="81" t="s">
+      <c r="D14" s="71" t="s">
         <v>263</v>
       </c>
-      <c r="E14" s="81" t="s">
+      <c r="E14" s="71" t="s">
         <v>264</v>
       </c>
-      <c r="F14" s="81" t="s">
+      <c r="F14" s="9" t="s">
         <v>265</v>
       </c>
       <c r="G14" s="3"/>
@@ -16309,22 +16309,22 @@
       <c r="AA14" s="3"/>
     </row>
     <row r="15" spans="1:27">
-      <c r="A15" s="80">
+      <c r="A15" s="70">
         <v>13</v>
       </c>
-      <c r="B15" s="81" t="s">
+      <c r="B15" s="71" t="s">
         <v>266</v>
       </c>
-      <c r="C15" s="81" t="s">
+      <c r="C15" s="71" t="s">
         <v>267</v>
       </c>
-      <c r="D15" s="81" t="s">
+      <c r="D15" s="71" t="s">
         <v>263</v>
       </c>
-      <c r="E15" s="81" t="s">
+      <c r="E15" s="71" t="s">
         <v>268</v>
       </c>
-      <c r="F15" s="81" t="s">
+      <c r="F15" s="9" t="s">
         <v>269</v>
       </c>
       <c r="G15" s="3"/>
@@ -44963,14 +44963,14 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="58"/>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="80" t="s">
         <v>229</v>
       </c>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
@@ -45077,14 +45077,14 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="62"/>
-      <c r="B13" s="77" t="s">
+      <c r="B13" s="81" t="s">
         <v>243</v>
       </c>
-      <c r="C13" s="69"/>
-      <c r="D13" s="69"/>
-      <c r="E13" s="69"/>
-      <c r="F13" s="69"/>
-      <c r="G13" s="69"/>
+      <c r="C13" s="73"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="73"/>
+      <c r="F13" s="73"/>
+      <c r="G13" s="73"/>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="8" t="s">

</xml_diff>